<commit_message>
Add Excel export images and update quotation rules
</commit_message>
<xml_diff>
--- a/products/Aluminum-Post-Wardrobe/Aluminum-Post-Wardrobe.xlsx
+++ b/products/Aluminum-Post-Wardrobe/Aluminum-Post-Wardrobe.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29400" windowHeight="12480"/>
+    <workbookView windowWidth="29400" windowHeight="12480" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="183">
   <si>
     <t>sku</t>
   </si>
@@ -174,6 +174,24 @@
     <t>customHeight</t>
   </si>
   <si>
+    <t>LZ-001-2</t>
+  </si>
+  <si>
+    <t>靠墙立柱</t>
+  </si>
+  <si>
+    <t>WALL-POST</t>
+  </si>
+  <si>
+    <t>post</t>
+  </si>
+  <si>
+    <t>LZ-001-2.glb</t>
+  </si>
+  <si>
+    <t>images/LZ-001-2.png</t>
+  </si>
+  <si>
     <t>LZ-001-4</t>
   </si>
   <si>
@@ -214,6 +232,51 @@
     <t>images/LZ-001-3.png</t>
   </si>
   <si>
+    <t>LZ-007-1</t>
+  </si>
+  <si>
+    <t>方立柱</t>
+  </si>
+  <si>
+    <t>POST-SQUARE</t>
+  </si>
+  <si>
+    <t>LZ-007-1.glb</t>
+  </si>
+  <si>
+    <t>images/LZ-007-1.png</t>
+  </si>
+  <si>
+    <t>LZ-007-2</t>
+  </si>
+  <si>
+    <t>靠墙方立柱</t>
+  </si>
+  <si>
+    <t>WALL-POST-SQUARE</t>
+  </si>
+  <si>
+    <t>LZ-007-2.glb</t>
+  </si>
+  <si>
+    <t>images/LZ-007-2png</t>
+  </si>
+  <si>
+    <t>LZ-007-3</t>
+  </si>
+  <si>
+    <t>方立柱调节脚</t>
+  </si>
+  <si>
+    <t>SQUARE-WALL-TOP-BRACKET</t>
+  </si>
+  <si>
+    <t>LZ-007-4</t>
+  </si>
+  <si>
+    <t>方立柱靠墙调节脚</t>
+  </si>
+  <si>
     <t>LZ-WOOD-SHELF</t>
   </si>
   <si>
@@ -568,16 +631,13 @@
     <t>condition</t>
   </si>
   <si>
-    <t>LZ-006-1</t>
-  </si>
-  <si>
     <t>led=true</t>
   </si>
   <si>
+    <t>connectionMode=ceiling</t>
+  </si>
+  <si>
     <t>connectionMode=wall</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> connectionMode=ceiling</t>
   </si>
   <si>
     <r>
@@ -638,10 +698,10 @@
     <t>defaultConnectionMode</t>
   </si>
   <si>
-    <t>celling</t>
-  </si>
-  <si>
-    <t>connectionMode</t>
+    <t>ceiling</t>
+  </si>
+  <si>
+    <t>connectionModeOptions</t>
   </si>
   <si>
     <t>wall/ceiling</t>
@@ -1677,12 +1737,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:T29"/>
+  <dimension ref="A1:T34"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="21.1964285714286" customWidth="1"/>
+    <col min="3" max="3" width="35.625" customWidth="1"/>
     <col min="4" max="4" width="21.8035714285714" customWidth="1"/>
     <col min="5" max="5" width="28.1964285714286" customWidth="1"/>
     <col min="6" max="6" width="23.6964285714286" customWidth="1"/>
@@ -1822,6 +1882,9 @@
       <c r="D3" s="2" t="s">
         <v>34</v>
       </c>
+      <c r="E3" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="H3" t="s">
         <v>24</v>
       </c>
@@ -1829,9 +1892,12 @@
         <v>25</v>
       </c>
       <c r="J3">
-        <v>34</v>
+        <v>169</v>
       </c>
       <c r="K3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L3" t="s">
         <v>35</v>
       </c>
       <c r="M3" t="b">
@@ -1844,10 +1910,10 @@
         <v>29</v>
       </c>
       <c r="P3" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="Q3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R3">
         <v>10</v>
@@ -1855,16 +1921,16 @@
     </row>
     <row r="4" ht="18" spans="1:20">
       <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" t="s">
         <v>38</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>39</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="H4" t="s">
         <v>24</v>
@@ -1873,22 +1939,22 @@
         <v>25</v>
       </c>
       <c r="J4">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="K4" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="M4" t="b">
         <v>1</v>
       </c>
       <c r="N4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="O4" t="s">
         <v>29</v>
       </c>
       <c r="P4" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -1897,71 +1963,65 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:20">
+    <row r="5" ht="18" spans="1:20">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J5">
+        <v>60</v>
+      </c>
+      <c r="K5" t="s">
+        <v>41</v>
+      </c>
+      <c r="M5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N5" t="s">
+        <v>47</v>
+      </c>
+      <c r="O5" t="s">
+        <v>29</v>
+      </c>
+      <c r="P5" t="s">
         <v>43</v>
       </c>
-      <c r="C5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G5">
-        <v>500</v>
-      </c>
-      <c r="H5" t="s">
-        <v>47</v>
-      </c>
-      <c r="I5" t="s">
-        <v>48</v>
-      </c>
-      <c r="K5" t="s">
-        <v>49</v>
-      </c>
-      <c r="L5" t="s">
-        <v>50</v>
-      </c>
-      <c r="M5" t="b">
+      <c r="Q5" t="b">
         <v>0</v>
       </c>
-      <c r="N5" t="s">
-        <v>51</v>
-      </c>
-      <c r="O5" t="s">
-        <v>52</v>
-      </c>
-      <c r="P5" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q5" t="b">
-        <v>1</v>
-      </c>
       <c r="R5">
-        <v>20</v>
-      </c>
-      <c r="S5" t="s">
-        <v>54</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" ht="18" spans="1:20">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>58</v>
+        <v>34</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="H6" t="s">
         <v>24</v>
@@ -1970,45 +2030,48 @@
         <v>25</v>
       </c>
       <c r="J6">
-        <v>50</v>
+        <v>169</v>
       </c>
       <c r="K6" t="s">
         <v>26</v>
       </c>
+      <c r="L6" t="s">
+        <v>51</v>
+      </c>
       <c r="M6" t="b">
         <v>1</v>
       </c>
       <c r="N6" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="O6" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="P6" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="Q6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6">
-        <v>20</v>
-      </c>
-      <c r="S6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" ht="18" spans="1:20">
       <c r="A7" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="C7" t="s">
-        <v>64</v>
-      </c>
-      <c r="D7" t="s">
-        <v>65</v>
+        <v>55</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="H7" t="s">
         <v>24</v>
@@ -2017,101 +2080,86 @@
         <v>25</v>
       </c>
       <c r="J7">
-        <v>20</v>
+        <v>169</v>
       </c>
       <c r="K7" t="s">
-        <v>66</v>
+        <v>26</v>
+      </c>
+      <c r="L7" t="s">
+        <v>56</v>
       </c>
       <c r="M7" t="b">
         <v>1</v>
       </c>
       <c r="N7" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="O7" t="s">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="P7" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="Q7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R7">
-        <v>90</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" ht="18" spans="1:20">
       <c r="A8" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D8" t="s">
-        <v>72</v>
-      </c>
-      <c r="E8" t="s">
-        <v>46</v>
-      </c>
-      <c r="G8">
-        <v>500</v>
+        <v>60</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="H8" t="s">
-        <v>73</v>
+        <v>24</v>
       </c>
       <c r="I8" t="s">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="J8">
-        <v>300</v>
+        <v>60</v>
       </c>
       <c r="K8" t="s">
-        <v>49</v>
-      </c>
-      <c r="L8" t="s">
-        <v>75</v>
+        <v>41</v>
       </c>
       <c r="M8" t="b">
         <v>1</v>
       </c>
-      <c r="N8" t="s">
-        <v>76</v>
-      </c>
       <c r="O8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P8" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q8" t="b">
+        <v>0</v>
+      </c>
+      <c r="R8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" ht="18" spans="1:20">
+      <c r="A9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" t="s">
         <v>60</v>
       </c>
-      <c r="P8" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q8" t="b">
-        <v>1</v>
-      </c>
-      <c r="R8">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20">
-      <c r="A9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B9" t="s">
-        <v>78</v>
-      </c>
-      <c r="C9" t="s">
-        <v>79</v>
-      </c>
-      <c r="D9" t="s">
-        <v>80</v>
-      </c>
-      <c r="E9" t="s">
-        <v>46</v>
-      </c>
-      <c r="G9" t="s">
-        <v>37</v>
+      <c r="D9" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="H9" t="s">
         <v>24</v>
@@ -2120,142 +2168,139 @@
         <v>25</v>
       </c>
       <c r="J9">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="K9" t="s">
-        <v>81</v>
-      </c>
-      <c r="L9" t="s">
-        <v>82</v>
+        <v>41</v>
       </c>
       <c r="M9" t="b">
         <v>1</v>
       </c>
-      <c r="N9" t="s">
-        <v>83</v>
-      </c>
       <c r="O9" t="s">
-        <v>84</v>
+        <v>29</v>
       </c>
       <c r="P9" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="Q9" t="b">
+        <v>0</v>
+      </c>
+      <c r="R9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20">
+      <c r="A10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G10">
+        <v>500</v>
+      </c>
+      <c r="H10" t="s">
+        <v>68</v>
+      </c>
+      <c r="I10" t="s">
+        <v>69</v>
+      </c>
+      <c r="K10" t="s">
+        <v>70</v>
+      </c>
+      <c r="L10" t="s">
+        <v>71</v>
+      </c>
+      <c r="M10" t="b">
+        <v>0</v>
+      </c>
+      <c r="N10" t="s">
+        <v>72</v>
+      </c>
+      <c r="O10" t="s">
+        <v>73</v>
+      </c>
+      <c r="P10" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q10" t="b">
         <v>1</v>
       </c>
-      <c r="R9">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" ht="18" spans="1:20">
-      <c r="A10" t="s">
-        <v>85</v>
-      </c>
-      <c r="B10" t="s">
-        <v>86</v>
-      </c>
-      <c r="C10" t="s">
-        <v>87</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="H10" t="s">
-        <v>24</v>
-      </c>
-      <c r="I10" t="s">
-        <v>25</v>
-      </c>
-      <c r="J10">
-        <v>3.5</v>
-      </c>
-      <c r="K10" t="s">
-        <v>35</v>
-      </c>
-      <c r="M10" t="b">
-        <v>1</v>
-      </c>
-      <c r="N10" t="s">
-        <v>89</v>
-      </c>
-      <c r="O10" t="s">
-        <v>84</v>
-      </c>
-      <c r="P10" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q10" t="b">
-        <v>0</v>
-      </c>
       <c r="R10">
-        <v>30</v>
+        <v>20</v>
+      </c>
+      <c r="S10" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="11" ht="18" spans="1:20">
       <c r="A11" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="G11">
-        <v>500</v>
+        <v>79</v>
       </c>
       <c r="H11" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="I11" t="s">
-        <v>48</v>
+        <v>25</v>
+      </c>
+      <c r="J11">
+        <v>50</v>
       </c>
       <c r="K11" t="s">
-        <v>35</v>
-      </c>
-      <c r="L11" t="s">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="M11" t="b">
+        <v>1</v>
+      </c>
+      <c r="N11" t="s">
+        <v>80</v>
+      </c>
+      <c r="O11" t="s">
+        <v>81</v>
+      </c>
+      <c r="P11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q11" t="b">
         <v>0</v>
       </c>
-      <c r="N11" t="s">
-        <v>95</v>
-      </c>
-      <c r="O11" t="s">
-        <v>96</v>
-      </c>
-      <c r="P11" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q11" t="b">
-        <v>1</v>
-      </c>
       <c r="R11">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="S11" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="12" ht="18" spans="1:20">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="B12" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="C12" t="s">
-        <v>99</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>100</v>
+        <v>85</v>
+      </c>
+      <c r="D12" t="s">
+        <v>86</v>
       </c>
       <c r="H12" t="s">
         <v>24</v>
@@ -2267,354 +2312,590 @@
         <v>20</v>
       </c>
       <c r="K12" t="s">
-        <v>35</v>
+        <v>87</v>
       </c>
       <c r="M12" t="b">
         <v>1</v>
       </c>
       <c r="N12" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="O12" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="P12" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
       </c>
       <c r="R12">
-        <v>40</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" ht="18" spans="1:20">
       <c r="A13" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="B13" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="C13" t="s">
-        <v>104</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>105</v>
+        <v>92</v>
+      </c>
+      <c r="D13" t="s">
+        <v>93</v>
       </c>
       <c r="E13" t="s">
-        <v>106</v>
-      </c>
-      <c r="F13">
-        <v>600</v>
+        <v>67</v>
       </c>
       <c r="G13">
         <v>500</v>
       </c>
       <c r="H13" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I13" t="s">
-        <v>25</v>
+        <v>95</v>
       </c>
       <c r="J13">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="K13" t="s">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="L13" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="M13" t="b">
         <v>1</v>
       </c>
       <c r="N13" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="O13" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="P13" t="s">
-        <v>37</v>
+        <v>74</v>
       </c>
       <c r="Q13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R13">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" ht="18" spans="1:20">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="B14" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C14" t="s">
-        <v>104</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
+      </c>
+      <c r="D14" t="s">
+        <v>101</v>
       </c>
       <c r="E14" t="s">
-        <v>106</v>
-      </c>
-      <c r="F14" s="2">
-        <v>700</v>
-      </c>
-      <c r="G14" s="2"/>
+        <v>67</v>
+      </c>
+      <c r="G14" t="s">
+        <v>43</v>
+      </c>
       <c r="H14" t="s">
-        <v>107</v>
+        <v>24</v>
       </c>
       <c r="I14" t="s">
         <v>25</v>
       </c>
       <c r="J14">
-        <v>298</v>
+        <v>13</v>
+      </c>
+      <c r="K14" t="s">
+        <v>102</v>
       </c>
       <c r="L14" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="M14" t="b">
         <v>1</v>
       </c>
       <c r="N14" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="O14" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="P14" t="s">
-        <v>37</v>
+        <v>74</v>
       </c>
       <c r="Q14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R14">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" ht="18" spans="1:20">
       <c r="A15" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B15" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C15" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="E15" t="s">
-        <v>106</v>
-      </c>
-      <c r="F15" s="2">
-        <v>800</v>
-      </c>
-      <c r="G15" s="2"/>
+        <v>109</v>
+      </c>
       <c r="H15" t="s">
-        <v>107</v>
+        <v>24</v>
       </c>
       <c r="I15" t="s">
         <v>25</v>
       </c>
       <c r="J15">
-        <v>308</v>
-      </c>
-      <c r="L15" t="s">
-        <v>111</v>
+        <v>3.5</v>
+      </c>
+      <c r="K15" t="s">
+        <v>41</v>
       </c>
       <c r="M15" t="b">
         <v>1</v>
       </c>
       <c r="N15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="O15" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="P15" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
       </c>
       <c r="R15">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" ht="18" spans="1:20">
       <c r="A16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B16" t="s">
         <v>112</v>
       </c>
-      <c r="B16" t="s">
-        <v>103</v>
-      </c>
       <c r="C16" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="E16" t="s">
-        <v>106</v>
-      </c>
-      <c r="F16" s="2">
-        <v>900</v>
-      </c>
-      <c r="G16" s="2"/>
+        <v>114</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G16">
+        <v>500</v>
+      </c>
       <c r="H16" t="s">
-        <v>107</v>
+        <v>68</v>
       </c>
       <c r="I16" t="s">
-        <v>25</v>
-      </c>
-      <c r="J16">
-        <v>318</v>
+        <v>69</v>
+      </c>
+      <c r="K16" t="s">
+        <v>41</v>
       </c>
       <c r="L16" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="M16" t="b">
+        <v>0</v>
+      </c>
+      <c r="N16" t="s">
+        <v>116</v>
+      </c>
+      <c r="O16" t="s">
+        <v>117</v>
+      </c>
+      <c r="P16" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q16" t="b">
         <v>1</v>
-      </c>
-      <c r="N16" t="s">
-        <v>109</v>
-      </c>
-      <c r="O16" t="s">
-        <v>96</v>
-      </c>
-      <c r="P16" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q16" t="b">
-        <v>0</v>
       </c>
       <c r="R16">
         <v>40</v>
       </c>
+      <c r="S16" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="17" ht="18" spans="1:18">
-      <c r="A17" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>114</v>
+      <c r="A17" t="s">
+        <v>118</v>
+      </c>
+      <c r="B17" t="s">
+        <v>119</v>
       </c>
       <c r="C17" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
+        <v>121</v>
+      </c>
       <c r="H17" t="s">
+        <v>24</v>
+      </c>
+      <c r="I17" t="s">
+        <v>25</v>
+      </c>
+      <c r="J17">
+        <v>20</v>
+      </c>
+      <c r="K17" t="s">
+        <v>41</v>
+      </c>
+      <c r="M17" t="b">
+        <v>1</v>
+      </c>
+      <c r="N17" t="s">
+        <v>122</v>
+      </c>
+      <c r="O17" t="s">
         <v>117</v>
       </c>
-      <c r="I17" t="s">
-        <v>118</v>
-      </c>
-      <c r="J17">
-        <v>26</v>
-      </c>
-      <c r="K17" t="s">
-        <v>119</v>
-      </c>
-      <c r="M17" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="N17" t="s">
-        <v>120</v>
-      </c>
-      <c r="O17" s="2" t="s">
-        <v>121</v>
-      </c>
       <c r="P17" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
       </c>
-      <c r="R17" s="2">
-        <v>50</v>
+      <c r="R17">
+        <v>40</v>
       </c>
     </row>
     <row r="18" ht="18" spans="1:18">
-      <c r="A18" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B18" s="2" t="s">
+      <c r="A18" t="s">
         <v>123</v>
       </c>
+      <c r="B18" t="s">
+        <v>124</v>
+      </c>
       <c r="C18" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+        <v>126</v>
+      </c>
+      <c r="E18" t="s">
+        <v>127</v>
+      </c>
+      <c r="F18">
+        <v>600</v>
+      </c>
+      <c r="G18">
+        <v>500</v>
+      </c>
       <c r="H18" t="s">
-        <v>126</v>
+        <v>128</v>
+      </c>
+      <c r="I18" t="s">
+        <v>25</v>
       </c>
       <c r="J18">
-        <v>39</v>
+        <v>288</v>
       </c>
       <c r="K18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M18" s="2" t="b">
+        <v>41</v>
+      </c>
+      <c r="L18" t="s">
+        <v>129</v>
+      </c>
+      <c r="M18" t="b">
         <v>1</v>
       </c>
       <c r="N18" t="s">
-        <v>127</v>
-      </c>
-      <c r="O18" s="2" t="s">
-        <v>121</v>
+        <v>130</v>
+      </c>
+      <c r="O18" t="s">
+        <v>117</v>
       </c>
       <c r="P18" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
       </c>
-      <c r="R18" s="2">
+      <c r="R18">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" ht="18" spans="1:18">
+      <c r="A19" t="s">
+        <v>131</v>
+      </c>
+      <c r="B19" t="s">
+        <v>124</v>
+      </c>
+      <c r="C19" t="s">
+        <v>125</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E19" t="s">
+        <v>127</v>
+      </c>
+      <c r="F19" s="2">
+        <v>700</v>
+      </c>
+      <c r="G19" s="2"/>
+      <c r="H19" t="s">
+        <v>128</v>
+      </c>
+      <c r="I19" t="s">
+        <v>25</v>
+      </c>
+      <c r="J19">
+        <v>298</v>
+      </c>
+      <c r="K19" t="s">
+        <v>41</v>
+      </c>
+      <c r="L19" t="s">
+        <v>131</v>
+      </c>
+      <c r="M19" t="b">
+        <v>1</v>
+      </c>
+      <c r="N19" t="s">
+        <v>130</v>
+      </c>
+      <c r="O19" t="s">
+        <v>117</v>
+      </c>
+      <c r="P19" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q19" t="b">
+        <v>0</v>
+      </c>
+      <c r="R19">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" ht="18" spans="1:18">
+      <c r="A20" t="s">
+        <v>132</v>
+      </c>
+      <c r="B20" t="s">
+        <v>124</v>
+      </c>
+      <c r="C20" t="s">
+        <v>125</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E20" t="s">
+        <v>127</v>
+      </c>
+      <c r="F20" s="2">
+        <v>800</v>
+      </c>
+      <c r="G20" s="2"/>
+      <c r="H20" t="s">
+        <v>128</v>
+      </c>
+      <c r="I20" t="s">
+        <v>25</v>
+      </c>
+      <c r="J20">
+        <v>308</v>
+      </c>
+      <c r="K20" t="s">
+        <v>41</v>
+      </c>
+      <c r="L20" t="s">
+        <v>132</v>
+      </c>
+      <c r="M20" t="b">
+        <v>1</v>
+      </c>
+      <c r="N20" t="s">
+        <v>130</v>
+      </c>
+      <c r="O20" t="s">
+        <v>117</v>
+      </c>
+      <c r="P20" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q20" t="b">
+        <v>0</v>
+      </c>
+      <c r="R20">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" ht="18" spans="1:18">
+      <c r="A21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B21" t="s">
+        <v>124</v>
+      </c>
+      <c r="C21" t="s">
+        <v>125</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E21" t="s">
+        <v>127</v>
+      </c>
+      <c r="F21" s="2">
+        <v>900</v>
+      </c>
+      <c r="G21" s="2"/>
+      <c r="H21" t="s">
+        <v>128</v>
+      </c>
+      <c r="I21" t="s">
+        <v>25</v>
+      </c>
+      <c r="J21">
+        <v>318</v>
+      </c>
+      <c r="K21" t="s">
+        <v>41</v>
+      </c>
+      <c r="L21" t="s">
+        <v>133</v>
+      </c>
+      <c r="M21" t="b">
+        <v>1</v>
+      </c>
+      <c r="N21" t="s">
+        <v>130</v>
+      </c>
+      <c r="O21" t="s">
+        <v>117</v>
+      </c>
+      <c r="P21" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q21" t="b">
+        <v>0</v>
+      </c>
+      <c r="R21">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" ht="18" spans="1:18">
+      <c r="A22" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C22" t="s">
+        <v>136</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" t="s">
+        <v>138</v>
+      </c>
+      <c r="I22" t="s">
+        <v>139</v>
+      </c>
+      <c r="J22">
+        <v>26</v>
+      </c>
+      <c r="K22" t="s">
+        <v>140</v>
+      </c>
+      <c r="M22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="N22" t="s">
+        <v>141</v>
+      </c>
+      <c r="O22" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="P22" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q22" t="b">
+        <v>0</v>
+      </c>
+      <c r="R22" s="2">
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:18">
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="1:18">
-      <c r="D21" s="2"/>
-    </row>
-    <row r="22" spans="1:18">
-      <c r="D22" s="2"/>
-    </row>
-    <row r="23" spans="1:18">
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-    </row>
-    <row r="24" spans="1:18">
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
+    <row r="23" ht="18" spans="1:18">
+      <c r="A23" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C23" t="s">
+        <v>145</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" t="s">
+        <v>147</v>
+      </c>
+      <c r="J23">
+        <v>39</v>
+      </c>
+      <c r="K23" t="s">
+        <v>41</v>
+      </c>
+      <c r="M23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="N23" t="s">
+        <v>148</v>
+      </c>
+      <c r="O23" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="P23" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q23" t="b">
+        <v>0</v>
+      </c>
+      <c r="R23" s="2">
+        <v>50</v>
+      </c>
     </row>
     <row r="25" spans="1:18">
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
     </row>
     <row r="26" spans="1:18">
       <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
     </row>
     <row r="27" spans="1:18">
       <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
     </row>
     <row r="28" spans="1:18">
       <c r="D28" s="2"/>
@@ -2623,6 +2904,26 @@
     <row r="29" spans="1:18">
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:18">
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:18">
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+    </row>
+    <row r="32" spans="1:18">
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+    </row>
+    <row r="33" spans="4:5">
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+    </row>
+    <row r="34" spans="4:5">
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
@@ -2634,9 +2935,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" outlineLevelCol="3"/>
   <cols>
+    <col min="1" max="1" width="23.6785714285714" customWidth="1"/>
     <col min="2" max="2" width="27.4017857142857" customWidth="1"/>
     <col min="3" max="3" width="22.0982142857143" customWidth="1"/>
     <col min="4" max="4" width="25.1071428571429" customWidth="1"/>
@@ -2644,24 +2946,24 @@
   <sheetData>
     <row r="1" ht="36" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="D1" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" ht="53" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="C2" s="2">
         <v>2</v>
@@ -2669,10 +2971,10 @@
     </row>
     <row r="3" ht="154" customHeight="1" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="C3" s="2">
         <v>2</v>
@@ -2680,10 +2982,10 @@
     </row>
     <row r="4" ht="154" customHeight="1" spans="1:4">
       <c r="A4" s="2" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="C4" s="2">
         <v>2</v>
@@ -2691,10 +2993,10 @@
     </row>
     <row r="5" ht="18" spans="1:4">
       <c r="A5" s="2" t="s">
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="C5" s="2">
         <v>2</v>
@@ -2702,10 +3004,10 @@
     </row>
     <row r="6" ht="53" spans="1:4">
       <c r="A6" s="2" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>97</v>
+        <v>118</v>
       </c>
       <c r="C6" s="2">
         <v>2</v>
@@ -2713,55 +3015,116 @@
     </row>
     <row r="7" ht="18" spans="1:4">
       <c r="A7" s="2" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="C7" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
-        <v>113</v>
-      </c>
-      <c r="B8" t="s">
-        <v>122</v>
-      </c>
-      <c r="C8">
+    <row r="8" ht="18" spans="1:4">
+      <c r="A8" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" ht="18" spans="1:4">
+      <c r="A9" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" ht="18" spans="1:4">
+      <c r="A10" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>134</v>
+      </c>
+      <c r="B11" t="s">
+        <v>143</v>
+      </c>
+      <c r="C11">
         <v>1</v>
       </c>
-      <c r="D8" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
+      <c r="D11" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
         <v>19</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
         <v>31</v>
       </c>
-      <c r="C9">
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13">
         <v>1</v>
       </c>
-      <c r="D9" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10">
+      <c r="D13" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14">
         <v>1</v>
       </c>
-      <c r="D10" t="s">
-        <v>135</v>
+      <c r="D14" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -2783,15 +3146,15 @@
   <sheetData>
     <row r="1" ht="18" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" ht="18" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>138</v>
+        <v>158</v>
       </c>
       <c r="B2" s="2">
         <v>500</v>
@@ -2799,7 +3162,7 @@
     </row>
     <row r="3" ht="18" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>139</v>
+        <v>159</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>24</v>
@@ -2807,31 +3170,31 @@
     </row>
     <row r="4" ht="18" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>141</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" ht="18" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>142</v>
+        <v>162</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" ht="18" spans="1:2">
       <c r="A6" t="s">
-        <v>144</v>
+        <v>164</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>145</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" ht="18" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
       <c r="B7" s="2" t="b">
         <v>0</v>
@@ -2839,18 +3202,18 @@
     </row>
     <row r="8" ht="18" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>147</v>
+        <v>167</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>148</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>149</v>
+        <v>169</v>
       </c>
       <c r="B9" t="s">
-        <v>150</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -2878,31 +3241,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>151</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" ht="18" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>152</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" ht="18" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>153</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s">
-        <v>153</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -2923,18 +3286,18 @@
   <sheetData>
     <row r="1" ht="18" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>154</v>
+        <v>174</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>155</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" ht="53" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>156</v>
+        <v>176</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>157</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -2954,15 +3317,15 @@
   <sheetData>
     <row r="1" ht="18" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>158</v>
+        <v>178</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>159</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" ht="18" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="B2" s="2">
         <v>30</v>
@@ -2970,7 +3333,7 @@
     </row>
     <row r="3" ht="18" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>161</v>
+        <v>181</v>
       </c>
       <c r="B3" s="2">
         <v>18</v>
@@ -2978,7 +3341,7 @@
     </row>
     <row r="4" ht="36" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>162</v>
+        <v>182</v>
       </c>
       <c r="B4" s="2">
         <v>28</v>

</xml_diff>